<commit_message>
Update AlgoComposition.xlsx from algo-helper
</commit_message>
<xml_diff>
--- a/AlgoComposition.xlsx
+++ b/AlgoComposition.xlsx
@@ -1,19 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2015" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2020" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2015" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2020" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2015'!$A$1:$E$51</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2020'!$A$1:$E$51</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -21,8 +18,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="0.000000000000000"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -34,23 +31,17 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="000F2744"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -58,24 +49,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -443,13 +432,6 @@
   </sheetPr>
   <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -479,1057 +461,1056 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>SNDK</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Sandisk Corporation</t>
         </is>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Broadcom</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>INTU</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Intuit</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>DELL</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Dell</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>MU</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Micron Technology</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>NVDA</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Palantir Technologies</t>
         </is>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>AMAT</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Applied Materials</t>
         </is>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>SHOP</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Shopify Inc.</t>
         </is>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>GRMN</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Garmin</t>
         </is>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="2" t="n">
         <v>45965</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Apple</t>
         </is>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>PEP</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="2" t="n">
         <v>46061</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>PepsiCo</t>
         </is>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>AMZN</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="2" t="n">
         <v>46073</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="2" t="n">
         <v>46140</v>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Amazon.com</t>
         </is>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>MU</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="2" t="n">
         <v>45993</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Micron Technology</t>
         </is>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>GOOG</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="2" t="n">
         <v>46073</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Google Inc.</t>
         </is>
       </c>
-      <c r="E16" s="4" t="n">
+      <c r="E16" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>ABNB</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="2" t="n">
         <v>46072</v>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Airbnb</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
+      <c r="E17" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>SNDK</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="2" t="n">
         <v>46061</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="2" t="n">
         <v>46072</v>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Sandisk Corporation</t>
         </is>
       </c>
-      <c r="E18" s="4" t="n">
+      <c r="E18" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="2" t="n">
         <v>45993</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="2" t="n">
         <v>46060</v>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Broadcom</t>
         </is>
       </c>
-      <c r="E19" s="4" t="n">
+      <c r="E19" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>TSLA</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="2" t="n">
         <v>46060</v>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Tesla</t>
         </is>
       </c>
-      <c r="E20" s="4" t="n">
+      <c r="E20" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>AZO</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="2" t="n">
         <v>45903</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C21" s="2" t="n">
         <v>45992</v>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>AutoZone</t>
         </is>
       </c>
-      <c r="E21" s="4" t="n">
+      <c r="E21" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>COST</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="2" t="n">
         <v>45903</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="2" t="n">
         <v>45992</v>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Costco Wholesale</t>
         </is>
       </c>
-      <c r="E22" s="4" t="n">
+      <c r="E22" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="2" t="n">
         <v>45964</v>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Home Depot</t>
         </is>
       </c>
-      <c r="E23" s="4" t="n">
+      <c r="E23" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>GRMN</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C24" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Garmin</t>
         </is>
       </c>
-      <c r="E24" s="4" t="n">
+      <c r="E24" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Mastercard</t>
         </is>
       </c>
-      <c r="E25" s="4" t="n">
+      <c r="E25" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>MELI</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>MercadoLibre</t>
         </is>
       </c>
-      <c r="E26" s="4" t="n">
+      <c r="E26" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>PEP</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>PepsiCo</t>
         </is>
       </c>
-      <c r="E27" s="4" t="n">
+      <c r="E27" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>APH</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="2" t="n">
         <v>45870</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" s="2" t="n">
         <v>45902</v>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Amphenol</t>
         </is>
       </c>
-      <c r="E28" s="4" t="n">
+      <c r="E28" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>HD</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" s="2" t="n">
         <v>45870</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C29" s="2" t="n">
         <v>45902</v>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Home Depot</t>
         </is>
       </c>
-      <c r="E29" s="4" t="n">
+      <c r="E29" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>INTU</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="2" t="n">
         <v>45869</v>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Intuit</t>
         </is>
       </c>
-      <c r="E30" s="4" t="n">
+      <c r="E30" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>NVDA</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" s="2" t="n">
         <v>45869</v>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="E31" s="4" t="n">
+      <c r="E31" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>APH</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Amphenol</t>
         </is>
       </c>
-      <c r="E32" s="4" t="n">
+      <c r="E32" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C33" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Deere</t>
         </is>
       </c>
-      <c r="E33" s="4" t="n">
+      <c r="E33" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C34" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Lowe's Companies</t>
         </is>
       </c>
-      <c r="E34" s="4" t="n">
+      <c r="E34" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>ORCL</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="2" t="n">
         <v>45811</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C35" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Oracle</t>
         </is>
       </c>
-      <c r="E35" s="4" t="n">
+      <c r="E35" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>LRCX</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C36" s="2" t="n">
         <v>45810</v>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Lam Research</t>
         </is>
       </c>
-      <c r="E36" s="4" t="n">
+      <c r="E36" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>LULU</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="2" t="n">
         <v>45692</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C37" s="2" t="n">
         <v>45777</v>
       </c>
-      <c r="D37" s="2" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Lululemon Athletica</t>
         </is>
       </c>
-      <c r="E37" s="4" t="n">
+      <c r="E37" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>TJX</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="C38" s="2" t="n">
         <v>45777</v>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>TJX Companies</t>
         </is>
       </c>
-      <c r="E38" s="4" t="n">
+      <c r="E38" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>WMT</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C39" s="2" t="n">
         <v>45777</v>
       </c>
-      <c r="D39" s="2" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Walmart</t>
         </is>
       </c>
-      <c r="E39" s="4" t="n">
+      <c r="E39" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="C40" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Apple</t>
         </is>
       </c>
-      <c r="E40" s="4" t="n">
+      <c r="E40" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>AMZN</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B41" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C41" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Amazon.com</t>
         </is>
       </c>
-      <c r="E41" s="4" t="n">
+      <c r="E41" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>GOOG</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B42" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="C42" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>Alphabet</t>
         </is>
       </c>
-      <c r="E42" s="4" t="n">
+      <c r="E42" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>MELI</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C43" s="3" t="n">
+      <c r="C43" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>MercadoLibre</t>
         </is>
       </c>
-      <c r="E43" s="4" t="n">
+      <c r="E43" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>PEP</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B44" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C44" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>PepsiCo</t>
         </is>
       </c>
-      <c r="E44" s="4" t="n">
+      <c r="E44" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>GRMN</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C45" s="3" t="n">
+      <c r="C45" s="2" t="n">
         <v>45691</v>
       </c>
-      <c r="D45" s="2" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Garmin</t>
         </is>
       </c>
-      <c r="E45" s="4" t="n">
+      <c r="E45" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>ABNB</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B46" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C46" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D46" s="2" t="inlineStr">
+      <c r="D46" t="inlineStr">
         <is>
           <t>Airbnb</t>
         </is>
       </c>
-      <c r="E46" s="4" t="n">
+      <c r="E46" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>DECK</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B47" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C47" s="3" t="n">
+      <c r="C47" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>Deckers Outdoor</t>
         </is>
       </c>
-      <c r="E47" s="4" t="n">
+      <c r="E47" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>QCOM</t>
         </is>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="C48" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>Qualcomm</t>
         </is>
       </c>
-      <c r="E48" s="4" t="n">
+      <c r="E48" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>STX</t>
         </is>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="C49" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D49" s="2" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Seagate Technology Hldgs</t>
         </is>
       </c>
-      <c r="E49" s="4" t="n">
+      <c r="E49" t="n">
         <v>0.142857142857143</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>PEP</t>
         </is>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B50" s="2" t="n">
         <v>46231</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C50" s="2" t="n">
         <v>46247</v>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="D50" t="inlineStr">
         <is>
           <t>PepsiCo</t>
         </is>
       </c>
-      <c r="E50" s="4" t="n">
+      <c r="E50" t="n">
         <v>0.1428571428571428</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>LRCX</t>
         </is>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B51" s="2" t="n">
         <v>46248</v>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C51" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Lam Research</t>
         </is>
       </c>
-      <c r="E51" s="4" t="n">
+      <c r="E51" t="n">
         <v>0.1428571428571428</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1542,13 +1523,6 @@
   </sheetPr>
   <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -1578,1057 +1552,1056 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" s="2" t="n">
         <v>46186</v>
       </c>
-      <c r="C2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>46247</v>
       </c>
-      <c r="D2" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="D2" t="n">
+        <v>0.142856</v>
+      </c>
+      <c r="E2" t="inlineStr">
         <is>
           <t>Broadcom</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>AMAT</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="2" t="n">
         <v>46175</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>46185</v>
       </c>
-      <c r="D3" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="D3" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>Applied Materials</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>SNDK</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B4" s="2" t="n">
         <v>46139</v>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D4" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="D4" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E4" t="inlineStr">
         <is>
           <t>Sandisk Corporation</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>APH</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B5" s="2" t="n">
         <v>46139</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>46230</v>
       </c>
-      <c r="D5" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="D5" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>Apollo</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>INTU</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B6" s="2" t="n">
         <v>46139</v>
       </c>
-      <c r="C6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D6" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="D6" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Intuit</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>MU</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B7" s="2" t="n">
         <v>45903</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D7" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="D7" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>Micron</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>NVDA</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
+      <c r="B8" s="2" t="n">
         <v>45965</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D8" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="D8" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>Nvidia</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
       </c>
-      <c r="B9" s="3" t="n">
+      <c r="B9" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D9" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="D9" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Palantir</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B10" s="3" t="n">
+      <c r="B10" s="2" t="n">
         <v>46139</v>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="2" t="n">
         <v>46174</v>
       </c>
-      <c r="D10" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="D10" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Broadcom</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>GRMN</t>
         </is>
       </c>
-      <c r="B11" s="3" t="n">
+      <c r="B11" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="2" t="n">
         <v>46138</v>
       </c>
-      <c r="D11" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D11" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>Garmin</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>SHOP</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n">
+      <c r="B12" s="2" t="n">
         <v>46091</v>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="2" t="n">
         <v>46138</v>
       </c>
-      <c r="D12" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D12" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Shopify Inc.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>AMZN</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n">
+      <c r="B13" s="2" t="n">
         <v>46077</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="2" t="n">
         <v>46138</v>
       </c>
-      <c r="D13" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="D13" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>Amazon Inc.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n">
+      <c r="B14" s="2" t="n">
         <v>46077</v>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="2" t="n">
         <v>46138</v>
       </c>
-      <c r="D14" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="D14" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>Apple Inc.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>GOOG</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n">
+      <c r="B15" s="2" t="n">
         <v>46077</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="2" t="n">
         <v>46090</v>
       </c>
-      <c r="D15" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="D15" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>Google Inc.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n">
+      <c r="B16" s="2" t="n">
         <v>45965</v>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="2" t="n">
         <v>46090</v>
       </c>
-      <c r="D16" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="D16" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E16" t="inlineStr">
         <is>
           <t>Broadcom</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>AMD</t>
         </is>
       </c>
-      <c r="B17" s="3" t="n">
+      <c r="B17" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="D17" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="D17" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>Advanced Micro Devices</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>ABNB</t>
         </is>
       </c>
-      <c r="B18" s="3" t="n">
+      <c r="B18" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="D18" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="D18" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>Airbnb</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>SNDK</t>
         </is>
       </c>
-      <c r="B19" s="3" t="n">
+      <c r="B19" s="2" t="n">
         <v>46061</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="2" t="n">
         <v>46076</v>
       </c>
-      <c r="D19" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="D19" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>Sandisk Corporation</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>HOOD</t>
         </is>
       </c>
-      <c r="B20" s="3" t="n">
+      <c r="B20" s="2" t="n">
         <v>46048</v>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="2" t="n">
         <v>46060</v>
       </c>
-      <c r="D20" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="D20" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>Robinhood Markets Inc</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>TSLA</t>
         </is>
       </c>
-      <c r="B21" s="3" t="n">
+      <c r="B21" s="2" t="n">
         <v>45993</v>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C21" s="2" t="n">
         <v>46047</v>
       </c>
-      <c r="D21" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="D21" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>Tesla</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>COST</t>
         </is>
       </c>
-      <c r="B22" s="3" t="n">
+      <c r="B22" s="2" t="n">
         <v>45903</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="2" t="n">
         <v>45992</v>
       </c>
-      <c r="D22" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="D22" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>Costco</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>APO</t>
         </is>
       </c>
-      <c r="B23" s="3" t="n">
+      <c r="B23" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="2" t="n">
         <v>45964</v>
       </c>
-      <c r="D23" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="D23" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>APO</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>AZO</t>
         </is>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B24" s="2" t="n">
         <v>45931</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C24" s="2" t="n">
         <v>45964</v>
       </c>
-      <c r="D24" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="D24" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>Autozone</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>APH</t>
         </is>
       </c>
-      <c r="B25" s="3" t="n">
+      <c r="B25" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D25" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="D25" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>APH</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>GRMN</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n">
+      <c r="B26" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D26" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="D26" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>Garmin</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
+      <c r="B27" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="C27" s="3" t="n">
+      <c r="C27" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D27" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="D27" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>Mastercard</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>MELI</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n">
+      <c r="B28" s="2" t="n">
         <v>45839</v>
       </c>
-      <c r="C28" s="3" t="n">
+      <c r="C28" s="2" t="n">
         <v>45930</v>
       </c>
-      <c r="D28" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="D28" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>Mercado Libre</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>KKR</t>
         </is>
       </c>
-      <c r="B29" s="3" t="n">
+      <c r="B29" s="2" t="n">
         <v>45870</v>
       </c>
-      <c r="C29" s="3" t="n">
+      <c r="C29" s="2" t="n">
         <v>45902</v>
       </c>
-      <c r="D29" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="D29" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>KKR</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>PEP</t>
         </is>
       </c>
-      <c r="B30" s="3" t="n">
+      <c r="B30" s="2" t="n">
         <v>45870</v>
       </c>
-      <c r="C30" s="3" t="n">
+      <c r="C30" s="2" t="n">
         <v>45902</v>
       </c>
-      <c r="D30" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="D30" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>Pepsi</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>INTU</t>
         </is>
       </c>
-      <c r="B31" s="3" t="n">
+      <c r="B31" s="2" t="n">
         <v>45692</v>
       </c>
-      <c r="C31" s="3" t="n">
+      <c r="C31" s="2" t="n">
         <v>45869</v>
       </c>
-      <c r="D31" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="D31" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>Intuit</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>NVDA</t>
         </is>
       </c>
-      <c r="B32" s="3" t="n">
+      <c r="B32" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C32" s="3" t="n">
+      <c r="C32" s="2" t="n">
         <v>45869</v>
       </c>
-      <c r="D32" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="D32" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E32" t="inlineStr">
         <is>
           <t>Nvidia</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>AJG</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
+      <c r="B33" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C33" s="3" t="n">
+      <c r="C33" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="D33" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="D33" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>AJG</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>NOW</t>
         </is>
       </c>
-      <c r="B34" s="3" t="n">
+      <c r="B34" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="C34" s="3" t="n">
+      <c r="C34" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="D34" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="D34" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>ServiceNow</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>ORCL</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
+      <c r="B35" s="2" t="n">
         <v>45811</v>
       </c>
-      <c r="C35" s="3" t="n">
+      <c r="C35" s="2" t="n">
         <v>45838</v>
       </c>
-      <c r="D35" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="D35" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>Oracle</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
-      <c r="B36" s="3" t="n">
+      <c r="B36" s="2" t="n">
         <v>45778</v>
       </c>
-      <c r="C36" s="3" t="n">
+      <c r="C36" s="2" t="n">
         <v>45810</v>
       </c>
-      <c r="D36" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="D36" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>DE</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B37" s="3" t="n">
+      <c r="B37" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C37" s="3" t="n">
+      <c r="C37" s="2" t="n">
         <v>45777</v>
       </c>
-      <c r="D37" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="D37" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>Broadcom</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" t="inlineStr">
         <is>
           <t>LULU</t>
         </is>
       </c>
-      <c r="B38" s="3" t="n">
+      <c r="B38" s="2" t="n">
         <v>45692</v>
       </c>
-      <c r="C38" s="3" t="n">
+      <c r="C38" s="2" t="n">
         <v>45777</v>
       </c>
-      <c r="D38" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="D38" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>Lululemon</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
+      <c r="A39" t="inlineStr">
         <is>
           <t>TJX</t>
         </is>
       </c>
-      <c r="B39" s="3" t="n">
+      <c r="B39" s="2" t="n">
         <v>45748</v>
       </c>
-      <c r="C39" s="3" t="n">
+      <c r="C39" s="2" t="n">
         <v>45777</v>
       </c>
-      <c r="D39" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="D39" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>TJX Companies</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
+      <c r="A40" t="inlineStr">
         <is>
           <t>AAPL</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B40" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C40" s="3" t="n">
+      <c r="C40" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D40" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="D40" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>Apple Inc.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr">
+      <c r="A41" t="inlineStr">
         <is>
           <t>AMZN</t>
         </is>
       </c>
-      <c r="B41" s="3" t="n">
+      <c r="B41" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C41" s="3" t="n">
+      <c r="C41" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D41" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="D41" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="inlineStr">
+      <c r="A42" t="inlineStr">
         <is>
           <t>GRMN</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B42" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C42" s="3" t="n">
+      <c r="C42" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D42" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="D42" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>Garmin</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
+      <c r="A43" t="inlineStr">
         <is>
           <t>MELI</t>
         </is>
       </c>
-      <c r="B43" s="3" t="n">
+      <c r="B43" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C43" s="3" t="n">
+      <c r="C43" s="2" t="n">
         <v>45747</v>
       </c>
-      <c r="D43" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="D43" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>Mercado Libre</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
+      <c r="A44" t="inlineStr">
         <is>
           <t>GOOG</t>
         </is>
       </c>
-      <c r="B44" s="3" t="n">
+      <c r="B44" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C44" s="3" t="n">
+      <c r="C44" s="2" t="n">
         <v>45691</v>
       </c>
-      <c r="D44" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="D44" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>Google Inc.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
       </c>
-      <c r="B45" s="3" t="n">
+      <c r="B45" s="2" t="n">
         <v>45660</v>
       </c>
-      <c r="C45" s="3" t="n">
+      <c r="C45" s="2" t="n">
         <v>45691</v>
       </c>
-      <c r="D45" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="D45" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>Palantir</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
+      <c r="A46" t="inlineStr">
         <is>
           <t>ABNB</t>
         </is>
       </c>
-      <c r="B46" s="3" t="n">
+      <c r="B46" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C46" s="3" t="n">
+      <c r="C46" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D46" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="D46" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>Airbnb</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
+      <c r="A47" t="inlineStr">
         <is>
           <t>AMD</t>
         </is>
       </c>
-      <c r="B47" s="3" t="n">
+      <c r="B47" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C47" s="3" t="n">
+      <c r="C47" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D47" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="D47" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E47" t="inlineStr">
         <is>
           <t>Advanced Micro Devices</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="inlineStr">
+      <c r="A48" t="inlineStr">
         <is>
           <t>APO</t>
         </is>
       </c>
-      <c r="B48" s="3" t="n">
+      <c r="B48" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C48" s="3" t="n">
+      <c r="C48" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D48" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="D48" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>APO</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="inlineStr">
+      <c r="A49" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="B49" s="3" t="n">
+      <c r="B49" s="2" t="n">
         <v>45653</v>
       </c>
-      <c r="C49" s="3" t="n">
+      <c r="C49" s="2" t="n">
         <v>45659</v>
       </c>
-      <c r="D49" s="4" t="n">
-        <v>0.142857142857143</v>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="D49" t="n">
+        <v>0.142857142857143</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>Visa</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" t="inlineStr">
         <is>
           <t>DELL</t>
         </is>
       </c>
-      <c r="B50" s="3" t="n">
+      <c r="B50" s="2" t="n">
         <v>46231</v>
       </c>
-      <c r="C50" s="3" t="n">
+      <c r="C50" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D50" s="4" t="n">
+      <c r="D50" t="n">
         <v>0.1428571428571428</v>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>DELL</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr">
+      <c r="A51" t="inlineStr">
         <is>
           <t>STX</t>
         </is>
       </c>
-      <c r="B51" s="3" t="n">
+      <c r="B51" s="2" t="n">
         <v>46248</v>
       </c>
-      <c r="C51" s="3" t="n">
+      <c r="C51" s="2" t="n">
         <v>55146</v>
       </c>
-      <c r="D51" s="4" t="n">
+      <c r="D51" t="n">
         <v>0.1428571428571428</v>
       </c>
-      <c r="E51" s="2" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>STX</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>